<commit_message>
fix: cap nhat cong thuc tinh chuan Circle K tu sheet SO, dong bo master data, web app, Excel, APK va backup
</commit_message>
<xml_diff>
--- a/Team_CamGiang_Report.xlsx
+++ b/Team_CamGiang_Report.xlsx
@@ -2161,7 +2161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F162"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2179,6 +2179,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -2394,6 +2395,7 @@
         <v>2270422</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
         <is>
@@ -2437,6 +2439,7 @@
         <v>2270422</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
@@ -2648,6 +2651,7 @@
         <v>2270422</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
@@ -2747,6 +2751,7 @@
         <v>26894000</v>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
@@ -3710,6 +3715,7 @@
         <v>1710740</v>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="36" t="inlineStr">
         <is>
@@ -5069,10 +5075,11 @@
         <v>1710740</v>
       </c>
     </row>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="36" t="inlineStr">
         <is>
-          <t>👤 Nguyễn Thị Thanh Thủy (38 cửa hàng CVS)</t>
+          <t>👤 Nguyễn Thị Thanh Thủy (39 cửa hàng CVS)</t>
         </is>
       </c>
       <c r="E115" s="37" t="inlineStr">
@@ -5172,6 +5179,21 @@
       <c r="A119" s="39" t="n">
         <v>103</v>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Thanh Thủy</t>
+        </is>
+      </c>
+      <c r="C119" s="44" t="inlineStr">
+        <is>
+          <t>Circle K</t>
+        </is>
+      </c>
+      <c r="D119" s="41" t="inlineStr">
+        <is>
+          <t>CVS_CIRCLEK.79.4260</t>
+        </is>
+      </c>
       <c r="E119" s="41" t="inlineStr">
         <is>
           <t>117/21, Thùy Vân, P.Vũng Tàu, TP.Hồ Chí Minh</t>
@@ -5183,35 +5205,20 @@
     </row>
     <row r="120">
       <c r="A120" s="39" t="n">
-        <v>104</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Thanh Thủy</t>
-        </is>
-      </c>
-      <c r="C120" s="44" t="inlineStr">
-        <is>
-          <t>Circle K</t>
-        </is>
-      </c>
-      <c r="D120" s="41" t="inlineStr">
-        <is>
-          <t>CVS_CIRCLEK.79.4267</t>
-        </is>
+        <v>103</v>
       </c>
       <c r="E120" s="41" t="inlineStr">
         <is>
-          <t>126A1, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>117/21, Thùy Vân, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F120" s="42" t="n">
-        <v>3497997</v>
+        <v>2985957</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="39" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -5225,21 +5232,21 @@
       </c>
       <c r="D121" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4252</t>
+          <t>CVS_CIRCLEK.79.4267</t>
         </is>
       </c>
       <c r="E121" s="41" t="inlineStr">
         <is>
-          <t>15, La Văn Cầu, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>126A1, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F121" s="42" t="n">
-        <v>2367117</v>
+        <v>3497997</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="39" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -5253,21 +5260,21 @@
       </c>
       <c r="D122" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4262</t>
+          <t>CVS_CIRCLEK.79.4252</t>
         </is>
       </c>
       <c r="E122" s="41" t="inlineStr">
         <is>
-          <t>152, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>15, La Văn Cầu, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F122" s="42" t="n">
-        <v>2726157</v>
+        <v>2367117</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="39" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -5281,21 +5288,21 @@
       </c>
       <c r="D123" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4265</t>
+          <t>CVS_CIRCLEK.79.4262</t>
         </is>
       </c>
       <c r="E123" s="41" t="inlineStr">
         <is>
-          <t>18, Nguyễn Trường Tộ, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>152, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F123" s="42" t="n">
-        <v>0</v>
+        <v>2726157</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="39" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -5309,21 +5316,21 @@
       </c>
       <c r="D124" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4268</t>
+          <t>CVS_CIRCLEK.79.4265</t>
         </is>
       </c>
       <c r="E124" s="41" t="inlineStr">
         <is>
-          <t>186, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>18, Nguyễn Trường Tộ, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F124" s="42" t="n">
-        <v>2372109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="39" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -5337,21 +5344,21 @@
       </c>
       <c r="D125" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4255</t>
+          <t>CVS_CIRCLEK.79.4268</t>
         </is>
       </c>
       <c r="E125" s="41" t="inlineStr">
         <is>
-          <t>205, Nam Kỳ Khởi Nghĩa, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>186, Hoàng Hoa Thám, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F125" s="42" t="n">
-        <v>2919501</v>
+        <v>2372109</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="39" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -5365,21 +5372,21 @@
       </c>
       <c r="D126" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4254</t>
+          <t>CVS_CIRCLEK.79.4255</t>
         </is>
       </c>
       <c r="E126" s="41" t="inlineStr">
         <is>
-          <t>26, Phan Văn Trị, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>205, Nam Kỳ Khởi Nghĩa, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F126" s="42" t="n">
-        <v>2066829</v>
+        <v>2919501</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="39" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -5393,21 +5400,21 @@
       </c>
       <c r="D127" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4269</t>
+          <t>CVS_CIRCLEK.79.4254</t>
         </is>
       </c>
       <c r="E127" s="41" t="inlineStr">
         <is>
-          <t>273, Lê Hồng Phong, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>26, Phan Văn Trị, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F127" s="42" t="n">
-        <v>3169317</v>
+        <v>2066829</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="39" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -5421,21 +5428,21 @@
       </c>
       <c r="D128" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4258</t>
+          <t>CVS_CIRCLEK.79.4269</t>
         </is>
       </c>
       <c r="E128" s="41" t="inlineStr">
         <is>
-          <t>4, Lê Lợi, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>273, Lê Hồng Phong, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F128" s="42" t="n">
-        <v>0</v>
+        <v>3169317</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="39" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -5449,21 +5456,21 @@
       </c>
       <c r="D129" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4259</t>
+          <t>CVS_CIRCLEK.79.4258</t>
         </is>
       </c>
       <c r="E129" s="41" t="inlineStr">
         <is>
-          <t>43, Thuỳ Vân, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>4, Lê Lợi, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F129" s="42" t="n">
-        <v>2367117</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="39" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -5477,21 +5484,21 @@
       </c>
       <c r="D130" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4256</t>
+          <t>CVS_CIRCLEK.79.4259</t>
         </is>
       </c>
       <c r="E130" s="41" t="inlineStr">
         <is>
-          <t>6, Quang Trung, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>43, Thuỳ Vân, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F130" s="42" t="n">
-        <v>3006909</v>
+        <v>2367117</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="39" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -5505,21 +5512,21 @@
       </c>
       <c r="D131" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4266</t>
+          <t>CVS_CIRCLEK.79.4256</t>
         </is>
       </c>
       <c r="E131" s="41" t="inlineStr">
         <is>
-          <t>78, Trần Hưng Đạo, P.Vũng Tàu, TP.Hồ Chí Minh</t>
+          <t>6, Quang Trung, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F131" s="42" t="n">
-        <v>0</v>
+        <v>3006909</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="39" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -5533,21 +5540,21 @@
       </c>
       <c r="D132" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4257</t>
+          <t>CVS_CIRCLEK.79.4266</t>
         </is>
       </c>
       <c r="E132" s="41" t="inlineStr">
         <is>
-          <t>Số 12 Khu Nhà DV 15 Tầng, Nguyễn Thái Học, P.Tam Thắng, TP.Hồ Chí Minh</t>
+          <t>78, Trần Hưng Đạo, P.Vũng Tàu, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F132" s="42" t="n">
-        <v>2066829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="39" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -5561,49 +5568,49 @@
       </c>
       <c r="D133" s="41" t="inlineStr">
         <is>
-          <t>CVS_CIRCLEK.79.4566</t>
+          <t>CVS_CIRCLEK.79.4257</t>
         </is>
       </c>
       <c r="E133" s="41" t="inlineStr">
         <is>
-          <t>Tầng 1, Chung Cư Kim Ngân, 275 Lê Hồng Phong, Phường Vũng Tàu, Thành phố Hồ Chí Minh, Việt Nam.</t>
+          <t>Số 12 Khu Nhà DV 15 Tầng, Nguyễn Thái Học, P.Tam Thắng, TP.Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F133" s="42" t="n">
-        <v>3833709</v>
+        <v>2066829</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="39" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
           <t>Nguyễn Thị Thanh Thủy</t>
         </is>
       </c>
-      <c r="C134" s="43" t="inlineStr">
-        <is>
-          <t>FamilyMart</t>
+      <c r="C134" s="44" t="inlineStr">
+        <is>
+          <t>Circle K</t>
         </is>
       </c>
       <c r="D134" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2639</t>
+          <t>CVS_CIRCLEK.79.4566</t>
         </is>
       </c>
       <c r="E134" s="41" t="inlineStr">
         <is>
-          <t>06, Hoàng Hoa Thám, , P.Vũng Tàu, Hồ Chí Minh</t>
+          <t>Tầng 1, Chung Cư Kim Ngân, 275 Lê Hồng Phong, Phường Vũng Tàu, Thành phố Hồ Chí Minh, Việt Nam.</t>
         </is>
       </c>
       <c r="F134" s="42" t="n">
-        <v>1930350</v>
+        <v>3833709</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="39" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -5617,21 +5624,21 @@
       </c>
       <c r="D135" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2636</t>
+          <t>CVS_FAMILYMART.79.2639</t>
         </is>
       </c>
       <c r="E135" s="41" t="inlineStr">
         <is>
-          <t>148, Hoàng Hoa Thám, , P.Vũng Tàu, Hồ Chí Minh</t>
+          <t>06, Hoàng Hoa Thám, , P.Vũng Tàu, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F135" s="42" t="n">
-        <v>2628150</v>
+        <v>1930350</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="39" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -5645,21 +5652,21 @@
       </c>
       <c r="D136" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2637</t>
+          <t>CVS_FAMILYMART.79.2636</t>
         </is>
       </c>
       <c r="E136" s="41" t="inlineStr">
         <is>
-          <t>171, Nam Kỳ Khởi Nghĩa, P.6, TP.Vũng Tàu, Bà Rịa Vũng Tàu</t>
+          <t>148, Hoàng Hoa Thám, , P.Vũng Tàu, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F136" s="42" t="n">
-        <v>2735700</v>
+        <v>2628150</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="39" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -5673,21 +5680,21 @@
       </c>
       <c r="D137" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2641</t>
+          <t>CVS_FAMILYMART.79.2637</t>
         </is>
       </c>
       <c r="E137" s="41" t="inlineStr">
         <is>
-          <t>26D, Lê Hồng Phong, , P.Tam Thắng, Hồ Chí Minh</t>
+          <t>171, Nam Kỳ Khởi Nghĩa, P.6, TP.Vũng Tàu, Bà Rịa Vũng Tàu</t>
         </is>
       </c>
       <c r="F137" s="42" t="n">
-        <v>3307200</v>
+        <v>2735700</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="39" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -5701,21 +5708,21 @@
       </c>
       <c r="D138" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2638</t>
+          <t>CVS_FAMILYMART.79.2641</t>
         </is>
       </c>
       <c r="E138" s="41" t="inlineStr">
         <is>
-          <t>48, Đồ Chiểu, , P.Vũng Tàu, Hồ Chí Minh</t>
+          <t>26D, Lê Hồng Phong, , P.Tam Thắng, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F138" s="42" t="n">
-        <v>692400</v>
+        <v>3307200</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="39" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -5729,21 +5736,21 @@
       </c>
       <c r="D139" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2640</t>
+          <t>CVS_FAMILYMART.79.2638</t>
         </is>
       </c>
       <c r="E139" s="41" t="inlineStr">
         <is>
-          <t>58, Trương Công Định, , P.Vũng Tàu, Hồ Chí Minh</t>
+          <t>48, Đồ Chiểu, , P.Vũng Tàu, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F139" s="42" t="n">
-        <v>2907600</v>
+        <v>692400</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="39" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -5757,49 +5764,49 @@
       </c>
       <c r="D140" s="41" t="inlineStr">
         <is>
-          <t>CVS_FAMILYMART.79.2635</t>
+          <t>CVS_FAMILYMART.79.2640</t>
         </is>
       </c>
       <c r="E140" s="41" t="inlineStr">
         <is>
-          <t>Số 816, Trần Phú, , P.Vũng Tàu, Hồ Chí Minh</t>
+          <t>58, Trương Công Định, , P.Vũng Tàu, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F140" s="42" t="n">
-        <v>1909500</v>
+        <v>2907600</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="39" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
           <t>Nguyễn Thị Thanh Thủy</t>
         </is>
       </c>
-      <c r="C141" s="40" t="inlineStr">
-        <is>
-          <t>GS25</t>
+      <c r="C141" s="43" t="inlineStr">
+        <is>
+          <t>FamilyMart</t>
         </is>
       </c>
       <c r="D141" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6654</t>
+          <t>CVS_FAMILYMART.79.2635</t>
         </is>
       </c>
       <c r="E141" s="41" t="inlineStr">
         <is>
-          <t>12 Trương Công Định, Phường 2, Vũng Tàu</t>
+          <t>Số 816, Trần Phú, , P.Vũng Tàu, Hồ Chí Minh</t>
         </is>
       </c>
       <c r="F141" s="42" t="n">
-        <v>2270422</v>
+        <v>1909500</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="39" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -5813,12 +5820,12 @@
       </c>
       <c r="D142" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6974</t>
+          <t>CVS_GS25.79.6654</t>
         </is>
       </c>
       <c r="E142" s="41" t="inlineStr">
         <is>
-          <t>28 thi sách, vũng tàu</t>
+          <t>12 Trương Công Định, Phường 2, Vũng Tàu</t>
         </is>
       </c>
       <c r="F142" s="42" t="n">
@@ -5827,7 +5834,7 @@
     </row>
     <row r="143">
       <c r="A143" s="39" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -5841,12 +5848,12 @@
       </c>
       <c r="D143" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6614</t>
+          <t>CVS_GS25.79.6974</t>
         </is>
       </c>
       <c r="E143" s="41" t="inlineStr">
         <is>
-          <t>41 Phó Đức Chính, Phường Thắng Tam, Vũng Tàu</t>
+          <t>28 thi sách, vũng tàu</t>
         </is>
       </c>
       <c r="F143" s="42" t="n">
@@ -5855,7 +5862,7 @@
     </row>
     <row r="144">
       <c r="A144" s="39" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -5869,12 +5876,12 @@
       </c>
       <c r="D144" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6965</t>
+          <t>CVS_GS25.79.6614</t>
         </is>
       </c>
       <c r="E144" s="41" t="inlineStr">
         <is>
-          <t>GS25 Hoàng Hoa Thám - Vũng Tàu</t>
+          <t>41 Phó Đức Chính, Phường Thắng Tam, Vũng Tàu</t>
         </is>
       </c>
       <c r="F144" s="42" t="n">
@@ -5883,7 +5890,7 @@
     </row>
     <row r="145">
       <c r="A145" s="39" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -5897,12 +5904,12 @@
       </c>
       <c r="D145" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6973</t>
+          <t>CVS_GS25.79.6965</t>
         </is>
       </c>
       <c r="E145" s="41" t="inlineStr">
         <is>
-          <t>GS25 Phan Văn Trị - Vũng Tàu</t>
+          <t>GS25 Hoàng Hoa Thám - Vũng Tàu</t>
         </is>
       </c>
       <c r="F145" s="42" t="n">
@@ -5911,7 +5918,7 @@
     </row>
     <row r="146">
       <c r="A146" s="39" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -5925,12 +5932,12 @@
       </c>
       <c r="D146" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6970</t>
+          <t>CVS_GS25.79.6973</t>
         </is>
       </c>
       <c r="E146" s="41" t="inlineStr">
         <is>
-          <t>Siêu thị GS-25 1A, Phó Đức Chính</t>
+          <t>GS25 Phan Văn Trị - Vũng Tàu</t>
         </is>
       </c>
       <c r="F146" s="42" t="n">
@@ -5939,7 +5946,7 @@
     </row>
     <row r="147">
       <c r="A147" s="39" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -5953,12 +5960,12 @@
       </c>
       <c r="D147" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6972</t>
+          <t>CVS_GS25.79.6970</t>
         </is>
       </c>
       <c r="E147" s="41" t="inlineStr">
         <is>
-          <t>Siêu thị GS-25 464, Trương Công Định</t>
+          <t>Siêu thị GS-25 1A, Phó Đức Chính</t>
         </is>
       </c>
       <c r="F147" s="42" t="n">
@@ -5967,7 +5974,7 @@
     </row>
     <row r="148">
       <c r="A148" s="39" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -5981,12 +5988,12 @@
       </c>
       <c r="D148" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6969</t>
+          <t>CVS_GS25.79.6972</t>
         </is>
       </c>
       <c r="E148" s="41" t="inlineStr">
         <is>
-          <t>Siêu thị GS-25 87, Thùy Vân</t>
+          <t>Siêu thị GS-25 464, Trương Công Định</t>
         </is>
       </c>
       <c r="F148" s="42" t="n">
@@ -5995,7 +6002,7 @@
     </row>
     <row r="149">
       <c r="A149" s="39" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -6009,12 +6016,12 @@
       </c>
       <c r="D149" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6968</t>
+          <t>CVS_GS25.79.6969</t>
         </is>
       </c>
       <c r="E149" s="41" t="inlineStr">
         <is>
-          <t>Siêu thị GS-25 Số 13, Trần Quý Cáp</t>
+          <t>Siêu thị GS-25 87, Thùy Vân</t>
         </is>
       </c>
       <c r="F149" s="42" t="n">
@@ -6023,7 +6030,7 @@
     </row>
     <row r="150">
       <c r="A150" s="39" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -6037,12 +6044,12 @@
       </c>
       <c r="D150" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6967</t>
+          <t>CVS_GS25.79.6968</t>
         </is>
       </c>
       <c r="E150" s="41" t="inlineStr">
         <is>
-          <t>Siêu thị GS-25 Số 53, Thùy Vân</t>
+          <t>Siêu thị GS-25 Số 13, Trần Quý Cáp</t>
         </is>
       </c>
       <c r="F150" s="42" t="n">
@@ -6051,7 +6058,7 @@
     </row>
     <row r="151">
       <c r="A151" s="39" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -6065,12 +6072,12 @@
       </c>
       <c r="D151" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6746</t>
+          <t>CVS_GS25.79.6967</t>
         </is>
       </c>
       <c r="E151" s="41" t="inlineStr">
         <is>
-          <t>Số 02-04 Đường Võ Thị Sáu, Phường 2, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
+          <t>Siêu thị GS-25 Số 53, Thùy Vân</t>
         </is>
       </c>
       <c r="F151" s="42" t="n">
@@ -6079,7 +6086,7 @@
     </row>
     <row r="152">
       <c r="A152" s="39" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -6093,12 +6100,12 @@
       </c>
       <c r="D152" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6764</t>
+          <t>CVS_GS25.79.6746</t>
         </is>
       </c>
       <c r="E152" s="41" t="inlineStr">
         <is>
-          <t>Số 51 đường Trưng Nhị (tầng 1 và tầng 2), Phường 1, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
+          <t>Số 02-04 Đường Võ Thị Sáu, Phường 2, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
         </is>
       </c>
       <c r="F152" s="42" t="n">
@@ -6107,7 +6114,7 @@
     </row>
     <row r="153">
       <c r="A153" s="39" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -6121,73 +6128,105 @@
       </c>
       <c r="D153" s="41" t="inlineStr">
         <is>
-          <t>CVS_GS25.79.6767</t>
+          <t>CVS_GS25.79.6764</t>
         </is>
       </c>
       <c r="E153" s="41" t="inlineStr">
         <is>
-          <t>Tầng 1 và tầng lửng căn hộ chung cư số LK-07, chung cư Vũng Tàu Center, Số 93 Lê Lợi, Phường Thắng Nhì, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
+          <t>Số 51 đường Trưng Nhị (tầng 1 và tầng 2), Phường 1, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
         </is>
       </c>
       <c r="F153" s="42" t="n">
         <v>2270422</v>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="36" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="39" t="n">
+        <v>137</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Thanh Thủy</t>
+        </is>
+      </c>
+      <c r="C154" s="40" t="inlineStr">
+        <is>
+          <t>GS25</t>
+        </is>
+      </c>
+      <c r="D154" s="41" t="inlineStr">
+        <is>
+          <t>CVS_GS25.79.6767</t>
+        </is>
+      </c>
+      <c r="E154" s="41" t="inlineStr">
+        <is>
+          <t>Tầng 1 và tầng lửng căn hộ chung cư số LK-07, chung cư Vũng Tàu Center, Số 93 Lê Lợi, Phường Thắng Nhì, Thành phố Vũng Tàu, Tỉnh Bà Rịa – Vũng Tàu</t>
+        </is>
+      </c>
+      <c r="F154" s="42" t="n">
+        <v>2270422</v>
+      </c>
+    </row>
+    <row r="155"/>
+    <row r="156">
+      <c r="A156" s="36" t="inlineStr">
         <is>
           <t>👤 Phạm Thị Kim Nhung (1 cửa hàng CVS)</t>
         </is>
       </c>
-      <c r="E155" s="37" t="inlineStr">
+      <c r="E156" s="37" t="inlineStr">
         <is>
           <t>TỔNG CVS:</t>
         </is>
       </c>
-      <c r="F155" s="38" t="n">
+      <c r="F156" s="38" t="n">
         <v>11234100</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="39" t="n">
+    <row r="157">
+      <c r="A157" s="39" t="n">
         <v>138</v>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B157" t="inlineStr">
         <is>
           <t>Phạm Thị Kim Nhung</t>
         </is>
       </c>
-      <c r="C156" s="48" t="inlineStr">
+      <c r="C157" s="48" t="inlineStr">
         <is>
           <t>Hoàng Đức Gia Kiệm</t>
         </is>
       </c>
-      <c r="D156" s="41" t="inlineStr">
+      <c r="D157" s="41" t="inlineStr">
         <is>
           <t>CVS_THECITY.75.1253</t>
         </is>
       </c>
-      <c r="E156" s="41" t="inlineStr">
+      <c r="E157" s="41" t="inlineStr">
         <is>
           <t>Số 166 Ấp Bạch Lâm 1, Xã Thống Nhất, Tỉnh Đồng Nai, Việt Nam</t>
         </is>
       </c>
-      <c r="F156" s="42" t="n">
+      <c r="F157" s="42" t="n">
         <v>11234100</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="49" t="inlineStr">
+    <row r="158"/>
+    <row r="159">
+      <c r="A159" s="49" t="inlineStr">
         <is>
           <t>🎯 TỔNG CVS TOÀN TEAM</t>
         </is>
       </c>
-      <c r="F158" s="50" t="n">
+      <c r="F159" s="50" t="n">
         <v>372666880</v>
       </c>
     </row>
-    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
     <row r="162"/>
+    <row r="163"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A159:D159"/>

</xml_diff>